<commit_message>
added custom rating types
</commit_message>
<xml_diff>
--- a/samples/template.xlsx
+++ b/samples/template.xlsx
@@ -64,175 +64,253 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dashboard Heading  The learner-facing heading on the section list, e.g. "Your Milestones".</t>
+          <t xml:space="preserve">  Dashboard Heading    The learner-facing heading on the section list, e.g. "Your Milestones".</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SECTIONS sheet: one row per section. Columns: Section ID, Title, Required (yes/no), Order.</t>
+          <t xml:space="preserve">  Allow PDF Download   yes or no. Shows learners a button to download a PDF of their responses.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QUESTIONS sheet: one row per question. Columns below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+          <t xml:space="preserve">                       Defaults to yes when the key is absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTIONS sheet: one row per section. Columns: Section ID, Title, Required (yes/no), Order.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Question columns:</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Section ID     Must match a Section ID from the Sections sheet.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">QUESTIONS sheet: one row per question. Columns below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Type           One of: short_text, long_text, yes_no, single_select, multiple_select, rating, checklist, numeric, url, datetime, acknowledgement, evidence_ref</t>
+          <t xml:space="preserve">Question columns:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prompt         The question text shown to the learner.</t>
+          <t xml:space="preserve">  Section ID     Must match a Section ID from the Sections sheet.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Required       yes or no. Only required questions gate section completion.</t>
+          <t xml:space="preserve">  Type           One of: short_text, long_text, yes_no, single_select, multiple_select, rating, checklist, numeric, url, datetime, acknowledgement, evidence_ref</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Options        Pipe-delimited choices for single_select / multiple_select / checklist, e.g. Yes | No | N/A</t>
+          <t xml:space="preserve">  Prompt         The question text shown to the learner.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 Prefix an option with * to mark it EXPECTED, e.g. Scope review | *Safety plan</t>
+          <t xml:space="preserve">  Required       yes or no. Only required questions gate section completion.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rating Scale   For rating questions only: 1-5  OR  Low|Medium|High</t>
+          <t xml:space="preserve">  Options        Pipe-delimited choices for single_select / multiple_select / checklist, e.g. Yes | No | N/A</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Min            For numeric questions. Inclusive lower bound, e.g. 4</t>
+          <t xml:space="preserve">                 Prefix an option with * to mark it EXPECTED, e.g. Scope review | *Safety plan</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Max            For numeric questions. Inclusive upper bound, e.g. 10</t>
+          <t xml:space="preserve">  Rating Scale   A scale id (agreement-5), a scale name (Agreement (5-point)),</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Whole Numbers  For numeric questions. yes to reject decimals.</t>
+          <t xml:space="preserve">                 explicit points (1=Strongly Agree | 2=Agree | 3=Neutral),</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Help Text      Optional guidance shown under the prompt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+          <t xml:space="preserve">                 bare labels (Low|Medium|High), or 1-5 for the numeric built-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Min            For numeric questions. Inclusive lower bound, e.g. 4</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completion rules:</t>
+          <t xml:space="preserve">  Max            For numeric questions. Inclusive upper bound, e.g. 10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A question is COMPLETE only when its response satisfies its requirement.</t>
+          <t xml:space="preserve">  Whole Numbers  For numeric questions. yes to reject decimals.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - checklist / multiple_select: the learner must select EVERY option marked with *.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - numeric: the value must fall within Min/Max (inclusive).</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  Help Text      Optional guidance shown under the prompt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - url: the value must be a valid http:// or https:// link.</t>
+          <t xml:space="preserve">Built-in rating scales:</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A question that has a response but fails its requirement is PARTIAL and does not count.</t>
+          <t xml:space="preserve">  numeric-5      1, 2, 3, 4, 5</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A section is COMPLETED only when every REQUIRED question in it is COMPLETE.</t>
+          <t xml:space="preserve">  agreement-5    Strongly Agree, Agree, Neutral, Disagree, Strongly Disagree</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A section where nothing is blank but a requirement is unmet shows as PARTIALLY COMPLETE.</t>
+          <t xml:space="preserve">  frequency-5    Always, Almost Always, Sometimes, Rarely, Never</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - The workbook reports "completed" only when every REQUIRED section is complete.</t>
+          <t xml:space="preserve">  confidence-3   Low, Medium, High</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manage your own scales on the Rating Scales screen in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completion rules:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A question is COMPLETE only when its response satisfies its requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - checklist / multiple_select: the learner must select EVERY option marked with *.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - numeric: the value must fall within Min/Max (inclusive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - url: the value must be a valid http:// or https:// link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - rating: the value must be one of the points in its scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A question that has a response but fails its requirement is PARTIAL and does not count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A section is COMPLETED only when every REQUIRED question in it is COMPLETE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A section where nothing is blank but a requirement is unmet shows as PARTIALLY COMPLETE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - The workbook reports "completed" only when every REQUIRED section is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t xml:space="preserve">  - evidence_ref records file metadata only; it never stores a file inside SCORM.</t>
         </is>
@@ -325,67 +403,79 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your observation workbook</t>
+          <t xml:space="preserve">Your Milestones</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navigation</t>
+          <t xml:space="preserve">Allow PDF Download</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">free</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completion Rule</t>
+          <t xml:space="preserve">Navigation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">all-required-sections</t>
+          <t xml:space="preserve">free</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report Success</t>
+          <t xml:space="preserve">Completion Rule</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">all-required-sections</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Course ID</t>
+          <t xml:space="preserve">Report Success</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ascend-ae-install-ride-along</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Course ID</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ascend-ae-install-ride-along</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Estimated Duration</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2-3 weeks</t>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 months</t>
         </is>
       </c>
     </row>
@@ -426,7 +516,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Install Team Meeting</t>
+          <t xml:space="preserve">Month 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -448,7 +538,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Install Manager Shadow</t>
+          <t xml:space="preserve">Month 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -470,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Install Technician Ride Along</t>
+          <t xml:space="preserve">Month 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -664,7 +754,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many install jobs did you review this week?</t>
+          <t xml:space="preserve">How many install jobs did you review this month?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -701,7 +791,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">How confident do you feel about the install handoff process?</t>
+          <t xml:space="preserve">The install handoff process was clearly explained.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -711,7 +801,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low|Medium|High</t>
+          <t xml:space="preserve">agreement-5</t>
         </is>
       </c>
     </row>
@@ -723,17 +813,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">long_text</t>
+          <t xml:space="preserve">rating</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe one thing you learned from the manager</t>
+          <t xml:space="preserve">How often did the team run a safety briefing?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frequency-5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add expected answers to more question types.
</commit_message>
<xml_diff>
--- a/samples/template.xlsx
+++ b/samples/template.xlsx
@@ -41,7 +41,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCORM Observation Workbook Builder - Excel Import Template</t>
+          <t xml:space="preserve">SOWB-It - Excel Import Template</t>
         </is>
       </c>
     </row>
@@ -85,232 +85,295 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">SECTIONS sheet: one row per section. Columns: Section ID, Title, Required (yes/no), Order.</t>
+          <t xml:space="preserve">SECTIONS sheet: one row per section. Columns: Section ID, Title, Required (yes/no), Order,</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">QUESTIONS sheet: one row per question. Columns below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+          <t xml:space="preserve">                Lock When Complete (yes/no).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lock When Complete   yes freezes the section once the learner completes it AND leaves it.</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Question columns:</t>
+          <t xml:space="preserve">                       They can still reopen and read it, but answers can no longer change,</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Section ID     Must match a Section ID from the Sections sheet.</t>
+          <t xml:space="preserve">                       and nothing in the SCO can unlock it. Defaults to no.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Type           One of: short_text, long_text, yes_no, single_select, multiple_select, rating, checklist, numeric, url, datetime, acknowledgement, evidence_ref</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Prompt         The question text shown to the learner.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">QUESTIONS sheet: one row per question. Columns below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Required       yes or no. Only required questions gate section completion.</t>
+          <t xml:space="preserve">Question columns:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Options        Pipe-delimited choices for single_select / multiple_select / checklist, e.g. Yes | No | N/A</t>
+          <t xml:space="preserve">  Section ID     Must match a Section ID from the Sections sheet.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 Prefix an option with * to mark it EXPECTED, e.g. Scope review | *Safety plan</t>
+          <t xml:space="preserve">  Type           One of: short_text, long_text, yes_no, single_select, multiple_select, rating, checklist, numeric, url, datetime, acknowledgement, evidence_ref</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rating Scale   A scale id (agreement-5), a scale name (Agreement (5-point)),</t>
+          <t xml:space="preserve">  Prompt         The question text shown to the learner.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 explicit points (1=Strongly Agree | 2=Agree | 3=Neutral),</t>
+          <t xml:space="preserve">  Required       yes or no. Only required questions gate section completion.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 bare labels (Low|Medium|High), or 1-5 for the numeric built-in.</t>
+          <t xml:space="preserve">  Options        Pipe-delimited choices for single_select / multiple_select / checklist, e.g. Yes | No | N/A</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Min            For numeric questions. Inclusive lower bound, e.g. 4</t>
+          <t xml:space="preserve">                 Prefix an option with * to mark it EXPECTED, e.g. Scope review | *Safety plan</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Max            For numeric questions. Inclusive upper bound, e.g. 10</t>
+          <t xml:space="preserve">                 On single_select, EXPECTED only sets correct / incorrect in the LMS report.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Whole Numbers  For numeric questions. yes to reject decimals.</t>
+          <t xml:space="preserve">  Rating Scale   A scale id (agreement-5), a scale name (Agreement (5-point)),</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Help Text      Optional guidance shown under the prompt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
+          <t xml:space="preserve">                 explicit points (1=Strongly Agree | 2=Agree | 3=Neutral),</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 bare labels (Low|Medium|High), or 1-5 for the numeric built-in.</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Built-in rating scales:</t>
+          <t xml:space="preserve">  Min            For numeric questions. Inclusive lower bound, e.g. 4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  numeric-5      1, 2, 3, 4, 5</t>
+          <t xml:space="preserve">  Max            For numeric questions. Inclusive upper bound, e.g. 10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  agreement-5    Strongly Agree, Agree, Neutral, Disagree, Strongly Disagree</t>
+          <t xml:space="preserve">  Whole Numbers  For numeric questions. yes to reject decimals.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  frequency-5    Always, Almost Always, Sometimes, Rarely, Never</t>
+          <t xml:space="preserve">  Expected       Optional, report-only. yes_no: yes or no. rating: a scale value or label,</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  confidence-3   Low, Medium, High</t>
+          <t xml:space="preserve">                 meaning that point or higher. Sets correct / incorrect in the LMS report;</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manage your own scales on the Rating Scales screen in the app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Completion rules:</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">                 any answer still completes the question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Help Text      Optional guidance shown under the prompt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A question is COMPLETE only when its response satisfies its requirement.</t>
+          <t xml:space="preserve">Built-in rating scales:</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - checklist / multiple_select: the learner must select EVERY option marked with *.</t>
+          <t xml:space="preserve">  numeric-5      1, 2, 3, 4, 5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - numeric: the value must fall within Min/Max (inclusive).</t>
+          <t xml:space="preserve">  agreement-5    Strongly Agree, Agree, Neutral, Disagree, Strongly Disagree</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - url: the value must be a valid http:// or https:// link.</t>
+          <t xml:space="preserve">  frequency-5    Always, Almost Always, Sometimes, Rarely, Never</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - rating: the value must be one of the points in its scale.</t>
+          <t xml:space="preserve">  confidence-3   Low, Medium, High</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A question that has a response but fails its requirement is PARTIAL and does not count.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - A section is COMPLETED only when every REQUIRED question in it is COMPLETE.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">Manage your own scales on the Rating Scales screen in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A section where nothing is blank but a requirement is unmet shows as PARTIALLY COMPLETE.</t>
+          <t xml:space="preserve">Completion rules:</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - The workbook reports "completed" only when every REQUIRED section is complete.</t>
+          <t xml:space="preserve">  - A question is COMPLETE only when its response satisfies its requirement.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - checklist / multiple_select: the learner must select EVERY option marked with *.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - numeric: the value must fall within Min/Max (inclusive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - url: the value must be a valid http:// or https:// link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - rating: the value must be one of the points in its scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A question that has a response but fails its requirement is PARTIAL and does not count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A section is COMPLETED only when every REQUIRED question in it is COMPLETE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A section where nothing is blank but a requirement is unmet shows as PARTIALLY COMPLETE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - The workbook reports "completed" only when every REQUIRED section is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A section with Lock When Complete freezes its answers once the learner completes it and leaves it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t xml:space="preserve">  - evidence_ref records file metadata only; it never stores a file inside SCORM.</t>
         </is>
@@ -507,6 +570,11 @@
           <t xml:space="preserve">Order</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock When Complete (yes/no)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,6 +597,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +624,11 @@
           <t xml:space="preserve">2</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -571,6 +649,11 @@
       <c r="D4" t="inlineStr">
         <is>
           <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
@@ -629,6 +712,11 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Expected</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Help Text</t>
         </is>
       </c>
@@ -654,7 +742,7 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use the date the meeting took place.</t>
         </is>
@@ -681,7 +769,7 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">Summarize scope, safety, and roles.</t>
         </is>
@@ -713,7 +801,7 @@
           <t xml:space="preserve">*Scope review | *Safety plan | Schedule | Customer expectations</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">Check all that apply.</t>
         </is>
@@ -772,7 +860,7 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve">Review at least four jobs.</t>
         </is>
@@ -804,6 +892,11 @@
           <t xml:space="preserve">agreement-5</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agree</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -853,6 +946,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -880,7 +978,7 @@
           <t xml:space="preserve">1-5</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">1 = low, 5 = high</t>
         </is>
@@ -907,7 +1005,7 @@
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t xml:space="preserve">Paste a SharePoint or Teams link starting with https://</t>
         </is>

</xml_diff>